<commit_message>
chore: checkpoint before modular upgrade
</commit_message>
<xml_diff>
--- a/Templates/钢筋安装检验批.xlsx
+++ b/Templates/钢筋安装检验批.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
-    <x:t>钢筋安装检验批质量验收记录</x:t>
+    <x:t>工程资料生成记录</x:t>
   </x:si>
   <x:si>
     <x:t>工程名称</x:t>
@@ -25,34 +25,82 @@
     <x:t>{{静态:工程名称}}</x:t>
   </x:si>
   <x:si>
+    <x:t>模板类型</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{静态:模板类型}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>建设单位</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{静态:建设单位}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>建设单位项目负责人</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{静态:建设单位项目负责人}}</x:t>
+  </x:si>
+  <x:si>
     <x:t>施工单位</x:t>
   </x:si>
   <x:si>
     <x:t>{{静态:施工单位}}</x:t>
   </x:si>
   <x:si>
+    <x:t>施工单位项目负责人</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{静态:施工单位项目负责人}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>设计单位</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{静态:设计单位}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>设计单位技术负责人</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{静态:设计单位技术负责人}}</x:t>
+  </x:si>
+  <x:si>
     <x:t>监理单位</x:t>
   </x:si>
   <x:si>
     <x:t>{{静态:监理单位}}</x:t>
   </x:si>
   <x:si>
-    <x:t>施工部位</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{静态:施工部位}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>分部工程</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{静态:分部工程}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>分项名称</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{静态:分项名称}}</x:t>
+    <x:t>总监理工程师</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{静态:监理单位总监理工程师}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>专业监理工程师</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{静态:监理单位专业监理工程师}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>检验批容量</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{静态:检验批容量}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>专业分包单位</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{静态:专业分包单位}}</x:t>
+  </x:si>
+  <x:si>
+    <x:t>第三方检测单位</x:t>
+  </x:si>
+  <x:si>
+    <x:t>{{静态:第三方检测单位}}</x:t>
   </x:si>
   <x:si>
     <x:t>施工日期</x:t>
@@ -65,24 +113,6 @@
   </x:si>
   <x:si>
     <x:t>{{静态:验收日期}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>主控项目</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{规范:主控项目表}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>一般项目</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{规范:一般项目表}}</x:t>
-  </x:si>
-  <x:si>
-    <x:t>允许偏差</x:t>
-  </x:si>
-  <x:si>
-    <x:t>{{规范:允许偏差表}}</x:t>
   </x:si>
   <x:si>
     <x:t>报验申请语</x:t>
@@ -503,7 +533,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F27"/>
+  <x:dimension ref="A1:F16"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="16.710625" style="0" customWidth="1"/>
@@ -592,36 +622,64 @@
       </x:c>
     </x:row>
     <x:row r="7" spans="1:6">
-      <x:c r="A7" s="3"/>
-      <x:c r="B7" s="3"/>
+      <x:c r="A7" s="3" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="s">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="C7" s="3"/>
-      <x:c r="D7" s="3"/>
-      <x:c r="E7" s="3"/>
+      <x:c r="D7" s="3" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E7" s="3" t="s">
+        <x:v>20</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" spans="1:6">
       <x:c r="A8" s="3" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B8" s="3"/>
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="s">
+        <x:v>22</x:v>
+      </x:c>
       <x:c r="C8" s="3"/>
-      <x:c r="D8" s="3"/>
-      <x:c r="E8" s="3"/>
+      <x:c r="D8" s="3" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="E8" s="3" t="s">
+        <x:v>24</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" spans="1:6">
       <x:c r="A9" s="3" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B9" s="3"/>
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="s">
+        <x:v>26</x:v>
+      </x:c>
       <x:c r="C9" s="3"/>
-      <x:c r="D9" s="3"/>
-      <x:c r="E9" s="3"/>
+      <x:c r="D9" s="3" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="E9" s="3" t="s">
+        <x:v>28</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" spans="1:6">
-      <x:c r="A10" s="3"/>
-      <x:c r="B10" s="3"/>
+      <x:c r="A10" s="3" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="s">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="C10" s="3"/>
-      <x:c r="D10" s="3"/>
-      <x:c r="E10" s="3"/>
+      <x:c r="D10" s="3" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="s">
+        <x:v>32</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" spans="1:6">
       <x:c r="A11" s="3"/>
@@ -631,16 +689,18 @@
       <x:c r="E11" s="3"/>
     </x:row>
     <x:row r="12" spans="1:6">
-      <x:c r="A12" s="3"/>
-      <x:c r="B12" s="3"/>
+      <x:c r="A12" s="3" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B12" s="3" t="s">
+        <x:v>34</x:v>
+      </x:c>
       <x:c r="C12" s="3"/>
       <x:c r="D12" s="3"/>
       <x:c r="E12" s="3"/>
     </x:row>
     <x:row r="13" spans="1:6">
-      <x:c r="A13" s="3" t="s">
-        <x:v>19</x:v>
-      </x:c>
+      <x:c r="A13" s="3"/>
       <x:c r="B13" s="3"/>
       <x:c r="C13" s="3"/>
       <x:c r="D13" s="3"/>
@@ -648,9 +708,11 @@
     </x:row>
     <x:row r="14" spans="1:6">
       <x:c r="A14" s="3" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B14" s="3"/>
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="s">
+        <x:v>36</x:v>
+      </x:c>
       <x:c r="C14" s="3"/>
       <x:c r="D14" s="3"/>
       <x:c r="E14" s="3"/>
@@ -663,107 +725,18 @@
       <x:c r="E15" s="3"/>
     </x:row>
     <x:row r="16" spans="1:6">
-      <x:c r="A16" s="3"/>
-      <x:c r="B16" s="3"/>
+      <x:c r="A16" s="3" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B16" s="3" t="s">
+        <x:v>38</x:v>
+      </x:c>
       <x:c r="C16" s="3"/>
-      <x:c r="D16" s="3"/>
-      <x:c r="E16" s="3"/>
-    </x:row>
-    <x:row r="17" spans="1:6">
-      <x:c r="A17" s="3"/>
-      <x:c r="B17" s="3"/>
-      <x:c r="C17" s="3"/>
-      <x:c r="D17" s="3"/>
-      <x:c r="E17" s="3"/>
-    </x:row>
-    <x:row r="18" spans="1:6">
-      <x:c r="A18" s="3" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B18" s="3"/>
-      <x:c r="C18" s="3"/>
-      <x:c r="D18" s="3"/>
-      <x:c r="E18" s="3"/>
-    </x:row>
-    <x:row r="19" spans="1:6">
-      <x:c r="A19" s="3" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B19" s="3"/>
-      <x:c r="C19" s="3"/>
-      <x:c r="D19" s="3"/>
-      <x:c r="E19" s="3"/>
-    </x:row>
-    <x:row r="20" spans="1:6">
-      <x:c r="A20" s="3"/>
-      <x:c r="B20" s="3"/>
-      <x:c r="C20" s="3"/>
-      <x:c r="D20" s="3"/>
-      <x:c r="E20" s="3"/>
-    </x:row>
-    <x:row r="21" spans="1:6">
-      <x:c r="A21" s="3"/>
-      <x:c r="B21" s="3"/>
-      <x:c r="C21" s="3"/>
-      <x:c r="D21" s="3"/>
-      <x:c r="E21" s="3"/>
-    </x:row>
-    <x:row r="22" spans="1:6">
-      <x:c r="A22" s="3"/>
-      <x:c r="B22" s="3"/>
-      <x:c r="C22" s="3"/>
-      <x:c r="D22" s="3"/>
-      <x:c r="E22" s="3"/>
-    </x:row>
-    <x:row r="23" spans="1:6">
-      <x:c r="A23" s="3" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="B23" s="3" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="C23" s="3"/>
-      <x:c r="D23" s="3"/>
-      <x:c r="E23" s="3"/>
-    </x:row>
-    <x:row r="24" spans="1:6">
-      <x:c r="A24" s="3"/>
-      <x:c r="B24" s="3"/>
-      <x:c r="C24" s="3"/>
-      <x:c r="D24" s="3"/>
-      <x:c r="E24" s="3"/>
-    </x:row>
-    <x:row r="25" spans="1:6">
-      <x:c r="A25" s="3" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="B25" s="3" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="C25" s="3"/>
-      <x:c r="D25" s="3"/>
-      <x:c r="E25" s="3"/>
-    </x:row>
-    <x:row r="26" spans="1:6">
-      <x:c r="A26" s="3"/>
-      <x:c r="B26" s="3"/>
-      <x:c r="C26" s="3"/>
-      <x:c r="D26" s="3"/>
-      <x:c r="E26" s="3"/>
-    </x:row>
-    <x:row r="27" spans="1:6">
-      <x:c r="A27" s="3" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B27" s="3" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C27" s="3"/>
-      <x:c r="D27" s="3" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="E27" s="3" t="s">
-        <x:v>30</x:v>
+      <x:c r="D16" s="3" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E16" s="3" t="s">
+        <x:v>40</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>